<commit_message>
Libretto Pietro: Fasi 1, 2 e 3
Aggiunte le tre voci scritte insieme a Manuel e Marco, datate 30/09/2026,
con una stima di 1 ora per la Fase 1 e 2,5 ore per ciascuna delle Fasi
2 e 3.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\AppData\Local\Temp\claude\C--Users-bulla-Documents-Ing-software-v1\c32cf868-ae9e-4ff3-a799-856eab5b1d43\scratchpad\out\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bulla\Documents\Ing-software-v1\docs\libretti\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDD6A234-32F2-4AD0-81E7-06AA076F7A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86EFF2B-C88A-4004-BBCD-D9EE54D9C4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2D331B93-E1FB-4C89-A78F-DFECF31FCEB5}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>Libretto delle attività</t>
   </si>
@@ -109,6 +109,33 @@
   </si>
   <si>
     <t>Se 'Fuori dalle settimane elencate' non è zero, ci sono voci con una data oltre l'ultima settimana: inserisci una riga sopra l'ultima settimana e copia le formule dalla riga precedente.</t>
+  </si>
+  <si>
+    <t>Fase 1 — Analisi del dominio</t>
+  </si>
+  <si>
+    <t>Con Manuel e Marco: analisi del dominio, 2 personas, Stakeholder Matrix e matrice di tracciabilità.</t>
+  </si>
+  <si>
+    <t>docs/fase-1-analisi-dominio.md</t>
+  </si>
+  <si>
+    <t>Fase 2 — Specifiche dei requisiti</t>
+  </si>
+  <si>
+    <t>Con Manuel e Marco: SRS Light con requisiti funzionali (MoSCoW), requisiti non funzionali e casi d'uso.</t>
+  </si>
+  <si>
+    <t>docs/fase-2-specifiche-requisiti.md</t>
+  </si>
+  <si>
+    <t>Fase 3 — Architettura e user flow</t>
+  </si>
+  <si>
+    <t>Con Manuel e Marco: casi d'uso in Mermaid, flusso delle schermate, architettura ad alto livello e diagrammi di sequenza.</t>
+  </si>
+  <si>
+    <t>docs/fase-3-architettura-user-flow.md</t>
   </si>
 </sst>
 </file>
@@ -276,119 +303,80 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -484,7 +472,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -503,7 +491,65 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFBF8F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1B2428"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -527,31 +573,12 @@
         </horizontal>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFBF8F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF1B2428"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Libretto" pivot="0" count="3" xr9:uid="{59739CDB-63D5-45D3-8730-D196FD7F67FA}">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
-      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="firstRowStripe" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -566,8 +593,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AA47867C-433E-4C7E-87B2-AAC0FCE68390}" name="Registro" displayName="Registro" ref="A8:E9" totalsRowShown="0" headerRowDxfId="2" dataDxfId="8">
-  <autoFilter ref="A8:E9" xr:uid="{AA47867C-433E-4C7E-87B2-AAC0FCE68390}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AA47867C-433E-4C7E-87B2-AAC0FCE68390}" name="Registro" displayName="Registro" ref="A8:E11" totalsRowShown="0" headerRowDxfId="8" dataDxfId="4">
+  <autoFilter ref="A8:E11" xr:uid="{AA47867C-433E-4C7E-87B2-AAC0FCE68390}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -575,11 +602,11 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C2248891-5FC5-425A-9EDE-392ECC4BF04A}" name="Data" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{373C6B70-9526-4B94-9B54-EAF5831EBA0A}" name="Attività" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{A7C421CB-05DB-4840-A964-AB66493E750B}" name="Ore" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{253DD084-FCA4-49D0-8D2F-FBD96DE74E29}" name="Descrizione" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{B340B777-29A7-4A97-BB16-FD91474C1774}" name="Risultato / file" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{C2248891-5FC5-425A-9EDE-392ECC4BF04A}" name="Data" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{373C6B70-9526-4B94-9B54-EAF5831EBA0A}" name="Attività" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{A7C421CB-05DB-4840-A964-AB66493E750B}" name="Ore" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{253DD084-FCA4-49D0-8D2F-FBD96DE74E29}" name="Descrizione" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{B340B777-29A7-4A97-BB16-FD91474C1774}" name="Risultato / file" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="Libretto" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -905,7 +932,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.59765625" style="1" customWidth="1"/>
@@ -942,7 +969,7 @@
       </c>
       <c r="C5" s="7">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -955,53 +982,97 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
+      <c r="A7" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="13.15" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
+    <row r="9" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="12">
+        <v>1</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="11">
+        <v>46295</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="12">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="C9:C11">
+    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9" xr:uid="{20ABBA9E-2AB5-4D0C-AC9C-86CF74ECBFC9}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data non valida" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." sqref="A9:A11" xr:uid="{20ABBA9E-2AB5-4D0C-AC9C-86CF74ECBFC9}">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9" xr:uid="{623F2EAD-18FD-4F42-BA32-BE4C81D73C78}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Ore non valide" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." promptTitle="Ore dedicate" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." sqref="C9:C11" xr:uid="{623F2EAD-18FD-4F42-BA32-BE4C81D73C78}">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1044,396 +1115,396 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
     </row>
     <row r="5" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="19">
+      <c r="A6" s="17">
         <v>46293</v>
       </c>
-      <c r="B6" s="20">
-        <f>A6+6</f>
+      <c r="B6" s="18">
+        <f t="shared" ref="B6:B21" si="0">A6+6</f>
         <v>46299</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="22">
+        <v>3</v>
+      </c>
+      <c r="D6" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A6,Registro[Data],"&lt;="&amp;B6)</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="22">
+        <v>6</v>
+      </c>
+      <c r="E6" s="20">
         <f>SUM(D$6:D6)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="23">
-        <f>A6+7</f>
+      <c r="A7" s="21">
+        <f t="shared" ref="A7:A21" si="1">A6+7</f>
         <v>46300</v>
       </c>
-      <c r="B7" s="23">
-        <f>A7+6</f>
+      <c r="B7" s="21">
+        <f t="shared" si="0"/>
         <v>46306</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A7,Registro[Data],"&lt;="&amp;B7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="23">
         <f>SUM(D$6:D7)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="20">
-        <f>A7+7</f>
+      <c r="A8" s="18">
+        <f t="shared" si="1"/>
         <v>46307</v>
       </c>
-      <c r="B8" s="20">
-        <f>A8+6</f>
+      <c r="B8" s="18">
+        <f t="shared" si="0"/>
         <v>46313</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="20">
         <f>SUM(D$6:D8)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="23">
-        <f>A8+7</f>
+      <c r="A9" s="21">
+        <f t="shared" si="1"/>
         <v>46314</v>
       </c>
-      <c r="B9" s="23">
-        <f>A9+6</f>
+      <c r="B9" s="21">
+        <f t="shared" si="0"/>
         <v>46320</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A9,Registro[Data],"&lt;="&amp;B9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="23">
         <f>SUM(D$6:D9)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="20">
-        <f>A9+7</f>
+      <c r="A10" s="18">
+        <f t="shared" si="1"/>
         <v>46321</v>
       </c>
-      <c r="B10" s="20">
-        <f>A10+6</f>
+      <c r="B10" s="18">
+        <f t="shared" si="0"/>
         <v>46327</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A10,Registro[Data],"&lt;="&amp;B10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="20">
         <f>SUM(D$6:D10)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="23">
-        <f>A10+7</f>
+      <c r="A11" s="21">
+        <f t="shared" si="1"/>
         <v>46328</v>
       </c>
-      <c r="B11" s="23">
-        <f>A11+6</f>
+      <c r="B11" s="21">
+        <f t="shared" si="0"/>
         <v>46334</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A11,Registro[Data],"&lt;="&amp;B11)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="23">
         <f>SUM(D$6:D11)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="20">
-        <f>A11+7</f>
+      <c r="A12" s="18">
+        <f t="shared" si="1"/>
         <v>46335</v>
       </c>
-      <c r="B12" s="20">
-        <f>A12+6</f>
+      <c r="B12" s="18">
+        <f t="shared" si="0"/>
         <v>46341</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A12,Registro[Data],"&lt;="&amp;B12)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="20">
         <f>SUM(D$6:D12)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="23">
-        <f>A12+7</f>
+      <c r="A13" s="21">
+        <f t="shared" si="1"/>
         <v>46342</v>
       </c>
-      <c r="B13" s="23">
-        <f>A13+6</f>
+      <c r="B13" s="21">
+        <f t="shared" si="0"/>
         <v>46348</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A13,Registro[Data],"&lt;="&amp;B13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="23">
         <f>SUM(D$6:D13)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="20">
-        <f>A13+7</f>
+      <c r="A14" s="18">
+        <f t="shared" si="1"/>
         <v>46349</v>
       </c>
-      <c r="B14" s="20">
-        <f>A14+6</f>
+      <c r="B14" s="18">
+        <f t="shared" si="0"/>
         <v>46355</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A14,Registro[Data],"&lt;="&amp;B14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="20">
         <f>SUM(D$6:D14)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="23">
-        <f>A14+7</f>
+      <c r="A15" s="21">
+        <f t="shared" si="1"/>
         <v>46356</v>
       </c>
-      <c r="B15" s="23">
-        <f>A15+6</f>
+      <c r="B15" s="21">
+        <f t="shared" si="0"/>
         <v>46362</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A15,Registro[Data],"&lt;="&amp;B15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="23">
         <f>SUM(D$6:D15)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="20">
-        <f>A15+7</f>
+      <c r="A16" s="18">
+        <f t="shared" si="1"/>
         <v>46363</v>
       </c>
-      <c r="B16" s="20">
-        <f>A16+6</f>
+      <c r="B16" s="18">
+        <f t="shared" si="0"/>
         <v>46369</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A16,Registro[Data],"&lt;="&amp;B16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="20">
         <f>SUM(D$6:D16)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="23">
-        <f>A16+7</f>
+      <c r="A17" s="21">
+        <f t="shared" si="1"/>
         <v>46370</v>
       </c>
-      <c r="B17" s="23">
-        <f>A17+6</f>
+      <c r="B17" s="21">
+        <f t="shared" si="0"/>
         <v>46376</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A17,Registro[Data],"&lt;="&amp;B17)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="23">
         <f>SUM(D$6:D17)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="20">
-        <f>A17+7</f>
+      <c r="A18" s="18">
+        <f t="shared" si="1"/>
         <v>46377</v>
       </c>
-      <c r="B18" s="20">
-        <f>A18+6</f>
+      <c r="B18" s="18">
+        <f t="shared" si="0"/>
         <v>46383</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A18,Registro[Data],"&lt;="&amp;B18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="20">
         <f>SUM(D$6:D18)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="23">
-        <f>A18+7</f>
+      <c r="A19" s="21">
+        <f t="shared" si="1"/>
         <v>46384</v>
       </c>
-      <c r="B19" s="23">
-        <f>A19+6</f>
+      <c r="B19" s="21">
+        <f t="shared" si="0"/>
         <v>46390</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="22">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="23">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A19,Registro[Data],"&lt;="&amp;B19)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="23">
         <f>SUM(D$6:D19)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="20">
-        <f>A19+7</f>
+      <c r="A20" s="18">
+        <f t="shared" si="1"/>
         <v>46391</v>
       </c>
-      <c r="B20" s="20">
-        <f>A20+6</f>
+      <c r="B20" s="18">
+        <f t="shared" si="0"/>
         <v>46397</v>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="19">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="20">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A20,Registro[Data],"&lt;="&amp;B20)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="20">
         <f>SUM(D$6:D20)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="26">
-        <f>A20+7</f>
+      <c r="A21" s="24">
+        <f t="shared" si="1"/>
         <v>46398</v>
       </c>
-      <c r="B21" s="26">
-        <f>A21+6</f>
+      <c r="B21" s="24">
+        <f t="shared" si="0"/>
         <v>46404</v>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="25">
         <f>COUNTIFS(Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="26">
         <f>SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A21,Registro[Data],"&lt;="&amp;B21)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="26">
         <f>SUM(D$6:D21)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31">
+      <c r="B22" s="28"/>
+      <c r="C22" s="29">
         <f>SUM(C6:C21)</f>
-        <v>0</v>
-      </c>
-      <c r="D22" s="32">
+        <v>3</v>
+      </c>
+      <c r="D22" s="30">
         <f>SUM(D6:D21)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="30"/>
+        <v>6</v>
+      </c>
+      <c r="E22" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
@@ -1441,9 +1512,9 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
-      <c r="D24" s="17">
+      <c r="D24" s="15">
         <f>SUM(Registro[Ore])</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.15" x14ac:dyDescent="0.4">
@@ -1452,19 +1523,19 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
-      <c r="D25" s="17">
+      <c r="D25" s="15">
         <f>D24-D22</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1472,7 +1543,7 @@
     <mergeCell ref="A26:E26"/>
   </mergeCells>
   <conditionalFormatting sqref="D25">
-    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="notEqual">
+    <cfRule type="cellIs" dxfId="6" priority="1" stopIfTrue="1" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Libretto Pietro: lettura documento D1
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016RNhFcM1MW3ZBovTFZi5y6
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
   <si>
     <t xml:space="preserve">Libretto delle attività</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t xml:space="preserve">docs/compiti.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lettura del documento D1 (Descrizione di Progetto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:14 – Aperto e letto il file D1-2026-V1.2.docx assegnato al gruppo: è il modello del documento di Requirements Engineering (progetto, RF, RNF, Use Case, User Story, mockup, traceability, modifiche).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D1-2026-V1.2.docx</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo delle ore</t>
@@ -327,19 +336,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -443,7 +452,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -586,8 +595,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A8:E12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A8:E13">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -781,7 +790,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.6"/>
@@ -802,12 +811,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -827,7 +836,7 @@
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">COUNTIFS(Registro[Attività],"&lt;&gt;",Registro[Ore],"")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -922,21 +931,36 @@
         <v>23</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C12">
+  <conditionalFormatting sqref="C9:C13">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." errorStyle="stop" errorTitle="Data non valida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A9:A12" type="date">
+    <dataValidation allowBlank="true" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." errorStyle="stop" errorTitle="Data non valida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A9:A13" type="date">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." errorStyle="stop" errorTitle="Ore non valide" operator="between" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." promptTitle="Ore dedicate" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9:C12" type="decimal">
+    <dataValidation allowBlank="true" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." errorStyle="stop" errorTitle="Ore non valide" operator="between" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." promptTitle="Ore dedicate" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9:C13" type="decimal">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -972,7 +996,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -982,7 +1006,7 @@
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -991,22 +1015,22 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="n">
         <v>46293</v>
       </c>
@@ -1027,7 +1051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="n">
         <f aca="false">A6+7</f>
         <v>46300</v>
@@ -1049,7 +1073,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="n">
         <f aca="false">A7+7</f>
         <v>46307</v>
@@ -1060,7 +1084,7 @@
       </c>
       <c r="C8" s="18" t="n">
         <f aca="false">COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
@@ -1071,7 +1095,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="n">
         <f aca="false">A8+7</f>
         <v>46314</v>
@@ -1093,7 +1117,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="n">
         <f aca="false">A9+7</f>
         <v>46321</v>
@@ -1115,7 +1139,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
         <f aca="false">A10+7</f>
         <v>46328</v>
@@ -1137,7 +1161,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="n">
         <f aca="false">A11+7</f>
         <v>46335</v>
@@ -1159,7 +1183,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
         <f aca="false">A12+7</f>
         <v>46342</v>
@@ -1181,7 +1205,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="n">
         <f aca="false">A13+7</f>
         <v>46349</v>
@@ -1203,7 +1227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
         <f aca="false">A14+7</f>
         <v>46356</v>
@@ -1225,7 +1249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="n">
         <f aca="false">A15+7</f>
         <v>46363</v>
@@ -1247,7 +1271,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
         <f aca="false">A16+7</f>
         <v>46370</v>
@@ -1269,7 +1293,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="n">
         <f aca="false">A17+7</f>
         <v>46377</v>
@@ -1291,7 +1315,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
         <f aca="false">A18+7</f>
         <v>46384</v>
@@ -1313,7 +1337,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="n">
         <f aca="false">A19+7</f>
         <v>46391</v>
@@ -1335,7 +1359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="n">
         <f aca="false">A20+7</f>
         <v>46398</v>
@@ -1359,12 +1383,12 @@
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="28" t="n">
         <f aca="false">SUM(C6:C21)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" s="29" t="n">
         <f aca="false">SUM(D6:D21)</f>
@@ -1374,7 +1398,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30"/>
@@ -1385,7 +1409,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B25" s="30"/>
       <c r="C25" s="30"/>
@@ -1396,7 +1420,7 @@
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>

</xml_diff>

<commit_message>
Aggiunto D1 finale test in presentazioni e libretto Pietro
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016RNhFcM1MW3ZBovTFZi5y6
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t xml:space="preserve">Libretto delle attività</t>
   </si>
@@ -105,6 +105,15 @@
   </si>
   <si>
     <t xml:space="preserve">D1-2026-V1.2.docx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salvataggio del documento D1 in presentazioni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:31 – Salvato il file D1 ricevuto dal gruppo nella cartella presentazioni con il nome «D1 finale test» e fatto il push su GitHub.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presentazioni/D1 finale test.docx</t>
   </si>
   <si>
     <t xml:space="preserve">Riepilogo delle ore</t>
@@ -595,8 +604,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A8:E13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A8:E14">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -790,7 +799,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.6"/>
@@ -836,7 +845,7 @@
       </c>
       <c r="C6" s="7" t="n">
         <f aca="false">COUNTIFS(Registro[Attività],"&lt;&gt;",Registro[Ore],"")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -946,21 +955,36 @@
         <v>26</v>
       </c>
     </row>
+    <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:E7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C13">
+  <conditionalFormatting sqref="C9:C14">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>($B9&lt;&gt;"")*($C9="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." errorStyle="stop" errorTitle="Data non valida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A9:A13" type="date">
+    <dataValidation allowBlank="true" error="Scrivi la data come gg/mm/aaaa, per esempio 14/10/2026." errorStyle="stop" errorTitle="Data non valida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="A9:A14" type="date">
       <formula1>46023</formula1>
       <formula2>47483</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." errorStyle="stop" errorTitle="Ore non valide" operator="between" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." promptTitle="Ore dedicate" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9:C13" type="decimal">
+    <dataValidation allowBlank="true" error="Scrivi le ore come numero tra 0 e 24 (1,5 = un'ora e mezza)." errorStyle="stop" errorTitle="Ore non valide" operator="between" prompt="Numero di ore, anche decimale: 1,5 = un'ora e mezza." promptTitle="Ore dedicate" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C9:C14" type="decimal">
       <formula1>0</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -996,7 +1020,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1006,7 +1030,7 @@
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -1015,19 +1039,19 @@
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1084,7 +1108,7 @@
       </c>
       <c r="C8" s="18" t="n">
         <f aca="false">COUNTIFS(Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">SUMIFS(Registro[Ore],Registro[Data],"&gt;="&amp;A8,Registro[Data],"&lt;="&amp;B8)</f>
@@ -1383,12 +1407,12 @@
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="28" t="n">
         <f aca="false">SUM(C6:C21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="29" t="n">
         <f aca="false">SUM(D6:D21)</f>
@@ -1398,7 +1422,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B24" s="30"/>
       <c r="C24" s="30"/>
@@ -1409,7 +1433,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B25" s="30"/>
       <c r="C25" s="30"/>
@@ -1420,7 +1444,7 @@
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>

</xml_diff>

<commit_message>
Elenco compiti più leggibile, senza le voci già fatte
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -349,8 +349,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E17" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A8:E17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E18" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A8:E18">
     <filterColumn colId="0" hiddenButton="1" showButton="1"/>
     <filterColumn colId="1" hiddenButton="1" showButton="1"/>
     <filterColumn colId="2" hiddenButton="1" showButton="1"/>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.06640625" defaultRowHeight="12.75"/>
   <cols>
     <col width="12.59765625" customWidth="1" style="1" min="1" max="1"/>
@@ -839,6 +839,29 @@
       <c r="E17" s="12" t="inlineStr">
         <is>
           <t>versione-corrente/frontend/src/stile.css, index.html, public/manifest.webmanifest</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38.25" customHeight="1">
+      <c r="A18" s="31" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Elenco compiti più leggibile, senza le voci già fatte</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Tolti i 42 compiti già fatti: restano i 19 da fare, divisi per area (requisiti aperti, da riverificare, documentazione, GDPR del titolare), con colonne separate per cosa fare e situazione attuale, filtri e riga fissa. Riepilogo aggiornato con la riga delle priorità non indicate. Fatto con l'aiuto di Claude (AI).</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>docs/compiti.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Benvenuto: presentazione di 15 foto di ieri e di oggi al posto della mappa
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -349,8 +349,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E18" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A8:E18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E19" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A8:E19">
     <filterColumn colId="0" hiddenButton="1" showButton="1"/>
     <filterColumn colId="1" hiddenButton="1" showButton="1"/>
     <filterColumn colId="2" hiddenButton="1" showButton="1"/>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.06640625" defaultRowHeight="12.75"/>
   <cols>
     <col width="12.59765625" customWidth="1" style="1" min="1" max="1"/>
@@ -862,6 +862,29 @@
       <c r="E18" s="12" t="inlineStr">
         <is>
           <t>docs/compiti.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38.25" customHeight="1">
+      <c r="A19" s="31" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Benvenuto: foto di Trento al posto della mappa</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Tolta la mappa dalla schermata di benvenuto e messa una presentazione di 15 foto, una alla volta a tutto riquadro, che cambiano da sole ogni 5 secondi con dissolvenza e un pulsante di pausa. Alternate 8 foto storiche (le stesse di "Dov'era?") e 7 attuali di affreschi e facciate scaricate da Wikimedia Commons con licenza libera; autore e licenza in piccolo su ogni foto. Testi in italiano, inglese e tedesco; parte ferma con "riduci movimento". Sistemati anche il testo scuro sul fondo petrolio nel tema chiaro e la larghezza sul telefono. Fatto con l'aiuto di Claude (AI).</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>versione-corrente/frontend/src/components/GalleriaBenvenuto.jsx, src/data/fotoBenvenuto.js, public/benvenuto/, src/pages/Benvenuto.jsx, src/stile.css</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pulsante satellite in alto a destra, solo icona
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -349,8 +349,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E19" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A8:E19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Registro" displayName="Registro" ref="A8:E20" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A8:E20">
     <filterColumn colId="0" hiddenButton="1" showButton="1"/>
     <filterColumn colId="1" hiddenButton="1" showButton="1"/>
     <filterColumn colId="2" hiddenButton="1" showButton="1"/>
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.06640625" defaultRowHeight="12.75"/>
   <cols>
     <col width="12.59765625" customWidth="1" style="1" min="1" max="1"/>
@@ -885,6 +885,29 @@
       <c r="E19" s="12" t="inlineStr">
         <is>
           <t>versione-corrente/frontend/src/components/GalleriaBenvenuto.jsx, src/data/fotoBenvenuto.js, public/benvenuto/, src/pages/Benvenuto.jsx, src/stile.css</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38.25" customHeight="1">
+      <c r="A20" s="31" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Pulsante satellite in alto a destra, solo icona</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Il pulsante con la scritta "Satellite" è ora un'icona quadrata in alto a destra della mappa: mostra il globo per passare al satellite e la mappa per tornare indietro, con colori petrolio e oro quando il satellite è attivo. Su telefono sta sotto ricerca e filtri e gli avvisi gli lasciano posto. Aggiunta l'icona al generatore e tolti i testi non più usati. Fatto con l'aiuto di Claude (AI).</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>versione-corrente/frontend/src/components/MappaLeaflet.jsx, src/stile.css, src/components/icone-svg.js</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cosa sto guardando: mappa dei luoghi al posto della fotocamera, con pannello sfumato
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/libretti/pietro-crea.xlsx
+++ b/docs/libretti/pietro-crea.xlsx
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Nella pagina "Cosa sto guardando?" (RF-06) si può ora scattare una foto o sceglierla dalla galleria. Si mostra la foto, si controlla da dove viene (scattata ora o dalla galleria, e se la posizione scritta nel file è vicina a chi la guarda) e si elencano i luoghi vicini al punto dello scatto. Lo scanner con posizione e bussola resta com'era. Testi in tre lingue, test della provenienza e prova nel browser anche con un file non valido. Fatto con l'aiuto di Claude (AI).</t>
+          <t>Nella pagina "Cosa sto guardando?" (RF-06) si può ora scattare una foto o sceglierla dalla galleria. Si mostra la foto, si controlla da dove viene (scattata ora o dalla galleria, e se la posizione scritta nel file è vicina a chi la guarda) e si elencano i luoghi vicini al punto dello scatto. Lo scanner con posizione e bussola resta com'era, ma al posto dell'anteprima della fotocamera c'è la mappa dei luoghi della guida attorno a te (con posizione, luoghi in vista e pulsante satellite) che sfuma nel pannello sotto su telefono; su desktop la mappa riempie la pagina e il pannello è una scheda di vetro sfumato sopra la mappa, con il pulsante satellite a sinistra. Testi in tre lingue, test della provenienza e prova nel browser anche con un file non valido. Fatto con l'aiuto di Claude (AI).</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>versione-corrente/frontend/src/pages/Inquadra.jsx, src/components/EsitoFoto.jsx, src/lib/provenienza.js, tests/frontend/provenienza.test.js</t>
+          <t>versione-corrente/frontend/src/pages/Inquadra.jsx, src/components/EsitoFoto.jsx, src/lib/provenienza.js, tests/frontend/provenienza.test.js, src/components/MappaLeaflet.jsx, src/stile.css</t>
         </is>
       </c>
     </row>

</xml_diff>